<commit_message>
fix: motor PWM pulled down
</commit_message>
<xml_diff>
--- a/hardware/docs/BOM_ordering.xlsx
+++ b/hardware/docs/BOM_ordering.xlsx
@@ -283,7 +283,7 @@
     <t>C154900</t>
   </si>
   <si>
-    <t>R1,R5,R6,R14,R19,R20, R_EN2</t>
+    <t>R1,R5,R6,R14,R16,R19,R20,R35,R36,R37,R38,R40,R41,R_EN2,</t>
   </si>
   <si>
     <t>RC0603FR-0710KL</t>
@@ -1653,7 +1653,7 @@
         <v>90</v>
       </c>
       <c r="B29" s="3">
-        <v>7.0</v>
+        <v>15.0</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>91</v>
@@ -1668,7 +1668,7 @@
         <v>0.0012</v>
       </c>
       <c r="G29" s="3">
-        <v>21.0</v>
+        <v>45.0</v>
       </c>
       <c r="H29" s="3">
         <v>100.0</v>

</xml_diff>